<commit_message>
3/9 Afternoon work on Post Race Analysis
</commit_message>
<xml_diff>
--- a/data/other/datadictionary.xlsx
+++ b/data/other/datadictionary.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jackguptill/Library/CloudStorage/OneDrive-Personal/Code/F1Fantasy/data/other/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jackguptill/Library/CloudStorage/OneDrive-Personal/Code/F1FantasyProject/data/other/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F56E9E7F-7149-D14F-9EC4-798B5D23ACAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2790DED6-E8CB-E14E-B838-CFB08BEE8CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{45E0BE48-3267-3742-B6D8-ABB2E8AD046B}"/>
   </bookViews>

</xml_diff>

<commit_message>
3/11 morning rerunning model and optimizer
</commit_message>
<xml_diff>
--- a/data/other/datadictionary.xlsx
+++ b/data/other/datadictionary.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jackguptill/Library/CloudStorage/OneDrive-Personal/Code/F1FantasyProject/data/other/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47AFB77E-B2D8-3046-83D8-2FBC277D62A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C3D28EF-12A3-8C4D-AB62-F3B7C86DC590}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4800" yWindow="500" windowWidth="28800" windowHeight="16380" xr2:uid="{45E0BE48-3267-3742-B6D8-ABB2E8AD046B}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="4" xr2:uid="{45E0BE48-3267-3742-B6D8-ABB2E8AD046B}"/>
   </bookViews>
   <sheets>
     <sheet name="PostRaceEval" sheetId="4" r:id="rId1"/>
     <sheet name="modelPerformance" sheetId="3" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
     <sheet name="driverdf" sheetId="1" r:id="rId4"/>
+    <sheet name="checklist" sheetId="5" r:id="rId5"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId5"/>
+    <externalReference r:id="rId6"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -64,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="183">
   <si>
     <t>features needed</t>
   </si>
@@ -550,6 +551,69 @@
   </si>
   <si>
     <t>Absolute Error</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>When</t>
+  </si>
+  <si>
+    <t>Post Race</t>
+  </si>
+  <si>
+    <t>Update Driver Points for past race</t>
+  </si>
+  <si>
+    <t>Update Constructor Points for past race</t>
+  </si>
+  <si>
+    <t>Update Current Week Driver Prices</t>
+  </si>
+  <si>
+    <t>Update Current Week Constructor Prices</t>
+  </si>
+  <si>
+    <t>Monday</t>
+  </si>
+  <si>
+    <t>Set 2026TeamConfig</t>
+  </si>
+  <si>
+    <t>verify current week lineup for the race</t>
+  </si>
+  <si>
+    <t>update Current Week Driver Roster</t>
+  </si>
+  <si>
+    <t>Run histDataClean</t>
+  </si>
+  <si>
+    <t>Verify current week within each of the core tables</t>
+  </si>
+  <si>
+    <t>Run driverLevelDataClean.ipynb</t>
+  </si>
+  <si>
+    <t>Verify hist_driver_points_df_v1.csv</t>
+  </si>
+  <si>
+    <t>Verify current_week_driver_points_df_v1.csv</t>
+  </si>
+  <si>
+    <t>Run driver Model</t>
+  </si>
+  <si>
+    <t>Verify driver_predictions_2026.csv</t>
+  </si>
+  <si>
+    <t>Change constructor model settings</t>
+  </si>
+  <si>
+    <t>run constructor model</t>
+  </si>
+  <si>
+    <t>run in week team optimizer</t>
   </si>
 </sst>
 </file>
@@ -3529,4 +3593,224 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8577ECF-3B0E-BA46-812D-AE5953F82593}">
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="43" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1" t="s">
+        <v>163</v>
+      </c>
+      <c r="D1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C3" t="s">
+        <v>164</v>
+      </c>
+      <c r="D3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>167</v>
+      </c>
+      <c r="C4" t="s">
+        <v>169</v>
+      </c>
+      <c r="D4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>168</v>
+      </c>
+      <c r="C5" t="s">
+        <v>169</v>
+      </c>
+      <c r="D5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>171</v>
+      </c>
+      <c r="C6" t="s">
+        <v>169</v>
+      </c>
+      <c r="D6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>172</v>
+      </c>
+      <c r="C7" t="s">
+        <v>169</v>
+      </c>
+      <c r="D7" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>173</v>
+      </c>
+      <c r="D8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>174</v>
+      </c>
+      <c r="D9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>175</v>
+      </c>
+      <c r="D10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>176</v>
+      </c>
+      <c r="D11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>178</v>
+      </c>
+      <c r="D13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>179</v>
+      </c>
+      <c r="D14" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>180</v>
+      </c>
+      <c r="D15" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>181</v>
+      </c>
+      <c r="D16" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>170</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
getting familiar with optimizer engine
</commit_message>
<xml_diff>
--- a/data/other/datadictionary.xlsx
+++ b/data/other/datadictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jackguptill/Library/CloudStorage/OneDrive-Personal/Code/F1FantasyProject/data/other/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C3D28EF-12A3-8C4D-AB62-F3B7C86DC590}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6ACB2F8-8D85-A74C-AB56-8467540D5B05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="4" xr2:uid="{45E0BE48-3267-3742-B6D8-ABB2E8AD046B}"/>
   </bookViews>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="188">
   <si>
     <t>features needed</t>
   </si>
@@ -556,9 +556,6 @@
     <t>Action</t>
   </si>
   <si>
-    <t>When</t>
-  </si>
-  <si>
     <t>Post Race</t>
   </si>
   <si>
@@ -577,9 +574,6 @@
     <t>Monday</t>
   </si>
   <si>
-    <t>Set 2026TeamConfig</t>
-  </si>
-  <si>
     <t>verify current week lineup for the race</t>
   </si>
   <si>
@@ -614,6 +608,27 @@
   </si>
   <si>
     <t>run in week team optimizer</t>
+  </si>
+  <si>
+    <t>Watch Race</t>
+  </si>
+  <si>
+    <t>Run post race anaysis</t>
+  </si>
+  <si>
+    <t>Sunday</t>
+  </si>
+  <si>
+    <t>Set 2026TeamConfig for week</t>
+  </si>
+  <si>
+    <t>Deadline</t>
+  </si>
+  <si>
+    <t>Do prior week notes</t>
+  </si>
+  <si>
+    <t>Figure out priorities for development</t>
   </si>
 </sst>
 </file>
@@ -3597,217 +3612,209 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8577ECF-3B0E-BA46-812D-AE5953F82593}">
-  <dimension ref="A1:D19"/>
+  <dimension ref="B1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="43" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>162</v>
       </c>
       <c r="C1" t="s">
-        <v>163</v>
+        <v>185</v>
       </c>
       <c r="D1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>1</v>
-      </c>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>164</v>
+      </c>
+      <c r="C3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
         <v>165</v>
       </c>
-      <c r="C2" t="s">
-        <v>164</v>
-      </c>
-      <c r="D2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>182</v>
+      </c>
+      <c r="C5" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>186</v>
+      </c>
+      <c r="C6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>187</v>
+      </c>
+      <c r="C7" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
         <v>166</v>
       </c>
-      <c r="C3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C8" t="s">
+        <v>168</v>
+      </c>
+      <c r="D8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
         <v>167</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C9" t="s">
+        <v>168</v>
+      </c>
+      <c r="D9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
         <v>169</v>
       </c>
-      <c r="D4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C10" t="s">
         <v>168</v>
       </c>
-      <c r="C5" t="s">
-        <v>169</v>
-      </c>
-      <c r="D5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="D10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>170</v>
+      </c>
+      <c r="C11" t="s">
+        <v>168</v>
+      </c>
+      <c r="D11" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
         <v>171</v>
       </c>
-      <c r="C6" t="s">
-        <v>169</v>
-      </c>
-      <c r="D6" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="D12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
         <v>172</v>
       </c>
-      <c r="C7" t="s">
-        <v>169</v>
-      </c>
-      <c r="D7" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="D13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
         <v>173</v>
       </c>
-      <c r="D8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="D14" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
         <v>174</v>
       </c>
-      <c r="D9" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="D15" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
         <v>175</v>
       </c>
-      <c r="D10" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="D16" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
         <v>176</v>
       </c>
-      <c r="D11" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="D17" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
         <v>177</v>
       </c>
-      <c r="D12" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="D18" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
         <v>178</v>
       </c>
-      <c r="D13" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="D19" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
         <v>179</v>
       </c>
-      <c r="D14" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="D20" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
         <v>180</v>
       </c>
-      <c r="D15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
         <v>181</v>
-      </c>
-      <c r="D16" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B19" t="s">
-        <v>170</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Elo Feature Added/Model updated and Ran
</commit_message>
<xml_diff>
--- a/data/other/datadictionary.xlsx
+++ b/data/other/datadictionary.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jackguptill/Library/CloudStorage/OneDrive-Personal/Code/F1FantasyProject/data/other/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F49755B1-F624-8D45-88C9-441FE48905B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF70BB7D-D3DC-3149-ABFB-9035F01C8585}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="4" xr2:uid="{45E0BE48-3267-3742-B6D8-ABB2E8AD046B}"/>
+    <workbookView xWindow="-28800" yWindow="-1260" windowWidth="28800" windowHeight="18000" activeTab="3" xr2:uid="{45E0BE48-3267-3742-B6D8-ABB2E8AD046B}"/>
   </bookViews>
   <sheets>
     <sheet name="PostRaceEval" sheetId="4" r:id="rId1"/>
     <sheet name="modelPerformance" sheetId="3" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
-    <sheet name="driverdf" sheetId="1" r:id="rId4"/>
-    <sheet name="checklist" sheetId="5" r:id="rId5"/>
+    <sheet name="driver model features" sheetId="1" r:id="rId4"/>
+    <sheet name="constructor_model_features" sheetId="6" r:id="rId5"/>
+    <sheet name="checklist" sheetId="5" r:id="rId6"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId6"/>
+    <externalReference r:id="rId7"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -65,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="188">
   <si>
     <t>features needed</t>
   </si>
@@ -250,18 +251,6 @@
     <t>Leak unless avg</t>
   </si>
   <si>
-    <t>Models</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Pre-Quali Model</t>
-  </si>
-  <si>
-    <t>Post-Quali Model</t>
-  </si>
-  <si>
     <t>race_dim, driver_points</t>
   </si>
   <si>
@@ -629,6 +618,18 @@
   </si>
   <si>
     <t>Figure out priorities for development</t>
+  </si>
+  <si>
+    <t>driver_elo</t>
+  </si>
+  <si>
+    <t>Week</t>
+  </si>
+  <si>
+    <t>log driver model results both pre and post tuning</t>
+  </si>
+  <si>
+    <t>points_std_last_5</t>
   </si>
 </sst>
 </file>
@@ -762,13 +763,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>507999</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>25400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>2624120</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>173020</xdr:colOff>
+      <xdr:row>45</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -806,13 +807,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>584199</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>1240090</xdr:colOff>
-      <xdr:row>27</xdr:row>
+      <xdr:colOff>1430590</xdr:colOff>
+      <xdr:row>34</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1226,16 +1227,16 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{34633587-BC6B-E54D-A700-556FFE11C3F8}" name="Table1" displayName="Table1" ref="A1:G55" totalsRowShown="0">
-  <autoFilter ref="A1:G55" xr:uid="{34633587-BC6B-E54D-A700-556FFE11C3F8}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{34633587-BC6B-E54D-A700-556FFE11C3F8}" name="Table1" displayName="Table1" ref="A1:G57" totalsRowShown="0">
+  <autoFilter ref="A1:G57" xr:uid="{34633587-BC6B-E54D-A700-556FFE11C3F8}">
     <filterColumn colId="1">
       <filters>
         <filter val="A,B"/>
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G55">
-    <sortCondition ref="A1:A55"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G57">
+    <sortCondition ref="A1:A57"/>
   </sortState>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{C13AFD3F-E9C5-5C4B-A50F-220F41424260}" name="Priority"/>
@@ -1562,28 +1563,28 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1" t="s">
+        <v>108</v>
+      </c>
+      <c r="D1" t="s">
+        <v>146</v>
+      </c>
+      <c r="E1" t="s">
         <v>111</v>
       </c>
-      <c r="B1" t="s">
-        <v>138</v>
-      </c>
-      <c r="C1" t="s">
-        <v>112</v>
-      </c>
-      <c r="D1" t="s">
-        <v>150</v>
-      </c>
-      <c r="E1" t="s">
-        <v>115</v>
-      </c>
       <c r="F1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H1" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
@@ -1591,10 +1592,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C2" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="G2">
         <f>VLOOKUP($B2,'[1]2026ConstructorPoints'!$A$1:$B$12,2,FALSE )</f>
@@ -1605,10 +1606,10 @@
         <v>96</v>
       </c>
       <c r="J2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="Q2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
@@ -1616,10 +1617,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C3" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="G3">
         <f>VLOOKUP($B3,'[1]2026ConstructorPoints'!$A$1:$B$12,2,FALSE )</f>
@@ -1630,7 +1631,7 @@
         <v>69</v>
       </c>
       <c r="J3" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="Q3" cm="1">
         <f t="array" ref="Q3">AVERAGE(ABS(Table2[Absolute Error]))</f>
@@ -1642,10 +1643,10 @@
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C4" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="G4">
         <f>VLOOKUP($B4,'[1]2026ConstructorPoints'!$A$1:$B$12,2,FALSE )</f>
@@ -1656,7 +1657,7 @@
         <v>35</v>
       </c>
       <c r="J4" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
@@ -1664,10 +1665,10 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C5" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="G5">
         <f>VLOOKUP($B5,'[1]2026ConstructorPoints'!$A$1:$B$12,2,FALSE )</f>
@@ -1678,7 +1679,7 @@
         <v>34</v>
       </c>
       <c r="J5" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
@@ -1686,16 +1687,16 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C6" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E6" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G6">
         <f>VLOOKUP($B6,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -1706,7 +1707,7 @@
         <v>50</v>
       </c>
       <c r="J6" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
@@ -1714,10 +1715,10 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C7" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="G7">
         <f>VLOOKUP($B7,'[1]2026ConstructorPoints'!$A$1:$B$12,2,FALSE )</f>
@@ -1733,10 +1734,10 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C8" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G8">
         <f>VLOOKUP($B8,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -1752,10 +1753,10 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C9" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G9">
         <f>VLOOKUP($B9,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -1771,10 +1772,10 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
+        <v>141</v>
+      </c>
+      <c r="C10" t="s">
         <v>145</v>
-      </c>
-      <c r="C10" t="s">
-        <v>149</v>
       </c>
       <c r="G10">
         <f>VLOOKUP($B10,'[1]2026ConstructorPoints'!$A$1:$B$12,2,FALSE )</f>
@@ -1790,10 +1791,10 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C11" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G11">
         <f>VLOOKUP($B11,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -1809,10 +1810,10 @@
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C12" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G12">
         <f>VLOOKUP($B12,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -1828,10 +1829,10 @@
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C13" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="G13">
         <f>VLOOKUP($B13,'[1]2026ConstructorPoints'!$A$1:$B$12,2,FALSE )</f>
@@ -1847,10 +1848,10 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C14" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G14">
         <f>VLOOKUP($B14,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -1866,16 +1867,16 @@
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C15" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="E15" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G15">
         <f>VLOOKUP($B15,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -1891,10 +1892,10 @@
         <v>1</v>
       </c>
       <c r="B16" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C16" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G16">
         <f>VLOOKUP($B16,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -1910,10 +1911,10 @@
         <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C17" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G17">
         <f>VLOOKUP($B17,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -1929,16 +1930,16 @@
         <v>1</v>
       </c>
       <c r="B18" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C18" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E18" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G18">
         <f>VLOOKUP($B18,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -1954,10 +1955,10 @@
         <v>1</v>
       </c>
       <c r="B19" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C19" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G19">
         <f>VLOOKUP($B19,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -1973,16 +1974,16 @@
         <v>1</v>
       </c>
       <c r="B20" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C20" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E20" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G20">
         <f>VLOOKUP($B20,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -1998,10 +1999,10 @@
         <v>1</v>
       </c>
       <c r="B21" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C21" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G21">
         <f>VLOOKUP($B21,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -2017,10 +2018,10 @@
         <v>1</v>
       </c>
       <c r="B22" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C22" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G22">
         <f>VLOOKUP($B22,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -2036,10 +2037,10 @@
         <v>1</v>
       </c>
       <c r="B23" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C23" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G23">
         <f>VLOOKUP($B23,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -2055,10 +2056,10 @@
         <v>1</v>
       </c>
       <c r="B24" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C24" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G24">
         <f>VLOOKUP($B24,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -2074,10 +2075,10 @@
         <v>1</v>
       </c>
       <c r="B25" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C25" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="G25">
         <f>VLOOKUP($B25,'[1]2026ConstructorPoints'!$A$1:$B$12,2,FALSE )</f>
@@ -2093,10 +2094,10 @@
         <v>1</v>
       </c>
       <c r="B26" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C26" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="G26">
         <f>VLOOKUP($B26,'[1]2026ConstructorPoints'!$A$1:$B$12,2,FALSE )</f>
@@ -2112,10 +2113,10 @@
         <v>1</v>
       </c>
       <c r="B27" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C27" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="G27">
         <f>VLOOKUP($B27,'[1]2026ConstructorPoints'!$A$1:$B$12,2,FALSE )</f>
@@ -2131,10 +2132,10 @@
         <v>1</v>
       </c>
       <c r="B28" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C28" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G28">
         <f>VLOOKUP($B28,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -2150,16 +2151,16 @@
         <v>1</v>
       </c>
       <c r="B29" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C29" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="E29" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G29">
         <f>VLOOKUP($B29,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -2175,10 +2176,10 @@
         <v>1</v>
       </c>
       <c r="B30" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C30" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G30">
         <f>VLOOKUP($B30,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -2194,16 +2195,16 @@
         <v>1</v>
       </c>
       <c r="B31" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C31" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E31" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G31">
         <f>VLOOKUP($B31,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -2219,10 +2220,10 @@
         <v>1</v>
       </c>
       <c r="B32" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C32" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G32">
         <f>VLOOKUP($B32,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -2238,10 +2239,10 @@
         <v>1</v>
       </c>
       <c r="B33" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C33" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="G33">
         <f>VLOOKUP($B33,'[1]2026DriverPoints'!$A$1:$B$23,2,FALSE )</f>
@@ -2257,10 +2258,10 @@
         <v>1</v>
       </c>
       <c r="B34" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C34" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="G34">
         <f>VLOOKUP($B34,'[1]2026ConstructorPoints'!$A$1:$B$12,2,FALSE )</f>
@@ -2281,341 +2282,662 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B754BE0A-32BD-0E49-8390-AEFF6E78917B}">
-  <dimension ref="B2:M14"/>
+  <dimension ref="B2:N25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="32.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.83203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.6640625" customWidth="1"/>
-    <col min="12" max="12" width="34.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.1640625" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="36" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.6640625" customWidth="1"/>
+    <col min="13" max="13" width="34.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="35.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>98</v>
+        <v>185</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>106</v>
       </c>
       <c r="L2" s="1" t="s">
         <v>102</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.2">
+        <v>98</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B3" s="7" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
-      <c r="G3" s="7">
+      <c r="G3" s="7"/>
+      <c r="H3" s="7">
         <v>12.356999999999999</v>
       </c>
-      <c r="H3" s="7">
+      <c r="I3" s="7">
         <v>16.077000000000002</v>
       </c>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
         <v>13.2</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>3.99</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>9.19</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>12.78</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>10.593999999999999</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>14.064</v>
-      </c>
-      <c r="I4">
-        <f>E4-G4</f>
-        <v>-1.4039999999999999</v>
       </c>
       <c r="J4">
         <f>F4-H4</f>
+        <v>-1.4039999999999999</v>
+      </c>
+      <c r="K4">
+        <f>G4-I4</f>
         <v>-1.2840000000000007</v>
       </c>
-      <c r="K4">
-        <f>C4-G4</f>
+      <c r="L4">
+        <f>D4-H4</f>
         <v>2.6059999999999999</v>
-      </c>
-      <c r="L4" s="6">
-        <f>($G$3-G4)/$G$3</f>
-        <v>0.14267216962045803</v>
       </c>
       <c r="M4" s="6">
         <f>($H$3-H4)/$H$3</f>
+        <v>0.14267216962045803</v>
+      </c>
+      <c r="N4" s="6">
+        <f>($I$3-I4)/$I$3</f>
         <v>0.12520992722522867</v>
       </c>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
         <v>11.288</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>1.0660000000000001</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>9.19</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>12.787000000000001</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>10.56</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>14.04</v>
       </c>
-      <c r="I5">
-        <f t="shared" ref="I5:I8" si="0">E5-G5</f>
+      <c r="J5">
+        <f t="shared" ref="J5:J13" si="0">F5-H5</f>
         <v>-1.370000000000001</v>
       </c>
-      <c r="J5">
-        <f t="shared" ref="J5:J8" si="1">F5-H5</f>
+      <c r="K5">
+        <f t="shared" ref="K5:K13" si="1">G5-I5</f>
         <v>-1.2529999999999983</v>
       </c>
-      <c r="K5">
-        <f t="shared" ref="K5:K8" si="2">C5-G5</f>
+      <c r="L5">
+        <f t="shared" ref="L5:L13" si="2">D5-H5</f>
         <v>0.72799999999999976</v>
       </c>
-      <c r="L5" s="6">
-        <f t="shared" ref="L5:L8" si="3">($G$3-G5)/$G$3</f>
+      <c r="M5" s="6">
+        <f t="shared" ref="M5:M13" si="3">($H$3-H5)/$H$3</f>
         <v>0.14542364651614462</v>
       </c>
-      <c r="M5" s="6">
-        <f t="shared" ref="M5:M8" si="4">($H$3-H5)/$H$3</f>
+      <c r="N5" s="6">
+        <f t="shared" ref="N5:N13" si="4">($I$3-I5)/$I$3</f>
         <v>0.12670274304907647</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
         <v>11.377000000000001</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>1.22</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>9.19</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>12.8</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>10.53</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>14.05</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <f t="shared" si="0"/>
         <v>-1.3399999999999999</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <f t="shared" si="1"/>
         <v>-1.25</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <f t="shared" si="2"/>
         <v>0.84700000000000131</v>
       </c>
-      <c r="L6" s="6">
+      <c r="M6" s="6">
         <f t="shared" si="3"/>
         <v>0.14785142024763293</v>
       </c>
-      <c r="M6" s="6">
+      <c r="N6" s="6">
         <f t="shared" si="4"/>
         <v>0.12608073645580647</v>
       </c>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
         <v>11.1</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>0.94499999999999995</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>9.1999999999999993</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>12.83</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>10.5</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>14.05</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <f t="shared" si="0"/>
         <v>-1.3000000000000007</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <f t="shared" si="1"/>
         <v>-1.2200000000000006</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <f t="shared" si="2"/>
         <v>0.59999999999999964</v>
       </c>
-      <c r="L7" s="6">
+      <c r="M7" s="6">
         <f t="shared" si="3"/>
         <v>0.1502791939791211</v>
       </c>
-      <c r="M7" s="6">
+      <c r="N7" s="6">
         <f t="shared" si="4"/>
         <v>0.12608073645580647</v>
       </c>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
         <v>10.43</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>0.98</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>6.58</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>9.31</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>10.66</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>14.41</v>
       </c>
-      <c r="I8" s="2">
+      <c r="J8" s="2">
         <f t="shared" si="0"/>
         <v>-4.08</v>
       </c>
-      <c r="J8" s="2">
+      <c r="K8" s="2">
         <f t="shared" si="1"/>
         <v>-5.0999999999999996</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <f t="shared" si="2"/>
         <v>-0.23000000000000043</v>
       </c>
-      <c r="L8" s="6">
+      <c r="M8" s="6">
         <f t="shared" si="3"/>
         <v>0.13733106741118389</v>
       </c>
-      <c r="M8" s="6">
+      <c r="N8" s="6">
         <f t="shared" si="4"/>
         <v>0.10368849909809053</v>
       </c>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B10" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>13.67</v>
+      </c>
+      <c r="E9">
+        <v>5.72</v>
+      </c>
+      <c r="F9">
+        <v>9.3699999999999992</v>
+      </c>
+      <c r="G9">
+        <v>12.97</v>
+      </c>
+      <c r="H9">
+        <v>10.210000000000001</v>
+      </c>
+      <c r="I9">
+        <v>13.67</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="0"/>
+        <v>-0.84000000000000163</v>
+      </c>
+      <c r="K9">
+        <f t="shared" si="1"/>
+        <v>-0.69999999999999929</v>
+      </c>
+      <c r="L9">
+        <f t="shared" si="2"/>
+        <v>3.4599999999999991</v>
+      </c>
+      <c r="M9" s="6">
+        <f t="shared" si="3"/>
+        <v>0.17374767338350722</v>
+      </c>
+      <c r="N9" s="6">
+        <f t="shared" si="4"/>
+        <v>0.14971698700006231</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <v>10.98</v>
+      </c>
+      <c r="E10">
+        <v>0.91100000000000003</v>
+      </c>
+      <c r="F10">
+        <v>9.4</v>
+      </c>
+      <c r="G10">
+        <v>12.99</v>
+      </c>
+      <c r="H10">
+        <v>10.14</v>
+      </c>
+      <c r="I10">
+        <v>13.45</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="0"/>
+        <v>-0.74000000000000021</v>
+      </c>
+      <c r="K10">
+        <f t="shared" si="1"/>
+        <v>-0.45999999999999908</v>
+      </c>
+      <c r="L10">
+        <f t="shared" si="2"/>
+        <v>0.83999999999999986</v>
+      </c>
+      <c r="M10" s="6">
+        <f t="shared" si="3"/>
+        <v>0.17941247875697977</v>
+      </c>
+      <c r="N10" s="6">
+        <f t="shared" si="4"/>
+        <v>0.16340113205199988</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <v>11.01</v>
+      </c>
+      <c r="E11">
+        <v>1.075</v>
+      </c>
+      <c r="F11">
+        <v>9.4</v>
+      </c>
+      <c r="G11">
+        <v>13.01</v>
+      </c>
+      <c r="H11">
+        <v>10.07</v>
+      </c>
+      <c r="I11">
+        <v>13.37</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="0"/>
+        <v>-0.66999999999999993</v>
+      </c>
+      <c r="K11">
+        <f t="shared" si="1"/>
+        <v>-0.35999999999999943</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="2"/>
+        <v>0.9399999999999995</v>
+      </c>
+      <c r="M11" s="6">
+        <f t="shared" si="3"/>
+        <v>0.1850772841304523</v>
+      </c>
+      <c r="N11" s="6">
+        <f t="shared" si="4"/>
+        <v>0.168377184798159</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>90</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12">
+        <v>10.9</v>
+      </c>
+      <c r="E12">
+        <v>0.93600000000000005</v>
+      </c>
+      <c r="F12">
+        <v>9.4499999999999993</v>
+      </c>
+      <c r="G12">
+        <v>13.06</v>
+      </c>
+      <c r="H12">
+        <v>10.050000000000001</v>
+      </c>
+      <c r="I12">
+        <v>13.35</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="0"/>
+        <v>-0.60000000000000142</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="1"/>
+        <v>-0.28999999999999915</v>
+      </c>
+      <c r="L12">
+        <f t="shared" si="2"/>
+        <v>0.84999999999999964</v>
+      </c>
+      <c r="M12" s="6">
+        <f t="shared" si="3"/>
+        <v>0.18669579995144442</v>
+      </c>
+      <c r="N12" s="6">
+        <f t="shared" si="4"/>
+        <v>0.16962119798469874</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13">
+        <v>10.38</v>
+      </c>
+      <c r="E13">
+        <v>0.9</v>
+      </c>
+      <c r="F13">
+        <v>6.57</v>
+      </c>
+      <c r="G13">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="H13">
+        <v>10.050000000000001</v>
+      </c>
+      <c r="I13">
+        <v>13.35</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="0"/>
+        <v>-3.4800000000000004</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="1"/>
+        <v>-4.0499999999999989</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="2"/>
+        <v>0.33000000000000007</v>
+      </c>
+      <c r="M13" s="6">
+        <f t="shared" si="3"/>
+        <v>0.18669579995144442</v>
+      </c>
+      <c r="N13" s="6">
+        <f t="shared" si="4"/>
+        <v>0.16962119798469874</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B17" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18">
         <v>9.6999999999999993</v>
       </c>
-      <c r="D11">
+      <c r="E18">
         <v>10.54</v>
       </c>
-      <c r="L11" s="5"/>
-    </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B12" t="s">
-        <v>95</v>
-      </c>
-      <c r="C12">
+      <c r="M18" s="5"/>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19">
         <v>9.6999999999999993</v>
       </c>
-      <c r="D12">
+      <c r="E19">
         <v>10.74</v>
       </c>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B13" t="s">
-        <v>94</v>
-      </c>
-      <c r="C13">
+    <row r="20" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
         <v>9.6999999999999993</v>
       </c>
-      <c r="D13">
+      <c r="E20">
         <v>10.723000000000001</v>
       </c>
     </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B14" t="s">
+    <row r="21" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>86</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="E21">
+        <v>10.61</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C22">
+        <v>2</v>
+      </c>
+      <c r="D22">
+        <v>10.01</v>
+      </c>
+      <c r="E22">
+        <v>9.9600000000000009</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23">
+        <v>2</v>
+      </c>
+      <c r="D23">
+        <v>10</v>
+      </c>
+      <c r="E23">
+        <v>9.94</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
         <v>90</v>
       </c>
-      <c r="C14">
-        <v>9.8000000000000007</v>
-      </c>
-      <c r="D14">
-        <v>10.61</v>
+      <c r="C24">
+        <v>2</v>
+      </c>
+      <c r="D24">
+        <v>9.9979999999999993</v>
+      </c>
+      <c r="E24">
+        <v>9.91</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>86</v>
+      </c>
+      <c r="C25">
+        <v>2</v>
+      </c>
+      <c r="D25">
+        <v>10.08</v>
+      </c>
+      <c r="E25">
+        <v>9.9990000000000006</v>
       </c>
     </row>
   </sheetData>
@@ -2631,23 +2953,23 @@
   <sheetData>
     <row r="3" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="H3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="H4" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.2">
       <c r="H5" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -2657,7 +2979,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B491CDF5-05FC-9645-86F5-29AA49D27163}">
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="34.1640625" bestFit="1" customWidth="1"/>
@@ -2668,7 +2990,7 @@
     <col min="11" max="11" width="15.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>52</v>
       </c>
@@ -2679,7 +3001,7 @@
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E1" t="s">
         <v>30</v>
@@ -2691,7 +3013,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2708,10 +3030,10 @@
         <v>39</v>
       </c>
       <c r="G2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2728,10 +3050,10 @@
         <v>39</v>
       </c>
       <c r="G3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1</v>
       </c>
@@ -2742,16 +3064,16 @@
         <v>2</v>
       </c>
       <c r="E4" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F4" t="s">
         <v>40</v>
       </c>
       <c r="G4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
@@ -2759,19 +3081,19 @@
         <v>55</v>
       </c>
       <c r="C5" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="E5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F5" t="s">
         <v>39</v>
       </c>
       <c r="G5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1</v>
       </c>
@@ -2779,19 +3101,19 @@
         <v>55</v>
       </c>
       <c r="C6" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E6" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F6" t="s">
         <v>39</v>
       </c>
       <c r="G6" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>1</v>
       </c>
@@ -2808,10 +3130,10 @@
         <v>40</v>
       </c>
       <c r="G7" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>1</v>
       </c>
@@ -2828,10 +3150,10 @@
         <v>39</v>
       </c>
       <c r="G8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>1</v>
       </c>
@@ -2849,10 +3171,10 @@
         <v>39</v>
       </c>
       <c r="G9" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>1</v>
       </c>
@@ -2869,30 +3191,30 @@
         <v>39</v>
       </c>
       <c r="G10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>1</v>
-      </c>
-      <c r="B11" t="s">
-        <v>55</v>
-      </c>
-      <c r="C11" t="s">
-        <v>81</v>
-      </c>
       <c r="E11" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F11" t="s">
         <v>39</v>
       </c>
       <c r="G11" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>1</v>
       </c>
@@ -2900,19 +3222,19 @@
         <v>55</v>
       </c>
       <c r="C12" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="E12" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F12" t="s">
         <v>39</v>
       </c>
       <c r="G12" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>1</v>
       </c>
@@ -2920,19 +3242,19 @@
         <v>55</v>
       </c>
       <c r="C13" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E13" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F13" t="s">
         <v>39</v>
       </c>
       <c r="G13" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>1</v>
       </c>
@@ -2940,19 +3262,19 @@
         <v>55</v>
       </c>
       <c r="C14" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E14" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F14" t="s">
         <v>39</v>
       </c>
       <c r="G14" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>1</v>
       </c>
@@ -2960,19 +3282,19 @@
         <v>55</v>
       </c>
       <c r="C15" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E15" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F15" t="s">
         <v>39</v>
       </c>
       <c r="G15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>1</v>
       </c>
@@ -2989,13 +3311,10 @@
         <v>53</v>
       </c>
       <c r="G16" t="s">
-        <v>67</v>
-      </c>
-      <c r="J16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>1</v>
       </c>
@@ -3012,16 +3331,10 @@
         <v>39</v>
       </c>
       <c r="G17" t="s">
-        <v>67</v>
-      </c>
-      <c r="J17" t="s">
-        <v>62</v>
-      </c>
-      <c r="K17" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>1</v>
       </c>
@@ -3038,16 +3351,10 @@
         <v>53</v>
       </c>
       <c r="G18" t="s">
-        <v>67</v>
-      </c>
-      <c r="J18" t="s">
-        <v>56</v>
-      </c>
-      <c r="K18" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>1</v>
       </c>
@@ -3061,10 +3368,10 @@
         <v>31</v>
       </c>
       <c r="G19" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>1</v>
       </c>
@@ -3072,16 +3379,16 @@
         <v>55</v>
       </c>
       <c r="C20" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E20" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="G20" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>1</v>
       </c>
@@ -3089,16 +3396,16 @@
         <v>55</v>
       </c>
       <c r="C21" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E21" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="G21" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>1</v>
       </c>
@@ -3115,21 +3422,24 @@
         <v>53</v>
       </c>
       <c r="G22" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>55</v>
       </c>
       <c r="C23" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+        <v>89</v>
+      </c>
+      <c r="G23" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>2</v>
       </c>
@@ -3137,13 +3447,13 @@
         <v>55</v>
       </c>
       <c r="C24" t="s">
-        <v>91</v>
-      </c>
-      <c r="E24" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+        <v>184</v>
+      </c>
+      <c r="G24" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>2</v>
       </c>
@@ -3151,87 +3461,87 @@
         <v>55</v>
       </c>
       <c r="C25" t="s">
+        <v>87</v>
+      </c>
+      <c r="E25" t="s">
+        <v>88</v>
+      </c>
+      <c r="G25" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>2</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" t="s">
         <v>12</v>
       </c>
-      <c r="E25" t="s">
-        <v>76</v>
-      </c>
-      <c r="F25" t="s">
-        <v>53</v>
-      </c>
-      <c r="G25" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A26">
-        <v>1</v>
-      </c>
-      <c r="B26" t="s">
-        <v>56</v>
-      </c>
-      <c r="C26" t="s">
-        <v>13</v>
-      </c>
       <c r="E26" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="F26" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="G26" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27">
-        <v>2</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>55</v>
+        <v>1</v>
+      </c>
+      <c r="B27" t="s">
+        <v>56</v>
       </c>
       <c r="C27" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E27" t="s">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="F27" t="s">
         <v>53</v>
       </c>
-      <c r="G27" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28">
-        <v>1</v>
-      </c>
-      <c r="B28" t="s">
+        <v>2</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" t="s">
+        <v>72</v>
+      </c>
+      <c r="F28" t="s">
+        <v>53</v>
+      </c>
+      <c r="G28" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>1</v>
+      </c>
+      <c r="B29" t="s">
         <v>56</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C29" t="s">
         <v>17</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E29" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A29">
-        <v>2</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C29" t="s">
-        <v>66</v>
-      </c>
-      <c r="E29" t="s">
-        <v>76</v>
-      </c>
-      <c r="G29" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>2</v>
       </c>
@@ -3239,41 +3549,45 @@
         <v>55</v>
       </c>
       <c r="C30" t="s">
-        <v>5</v>
+        <v>62</v>
       </c>
       <c r="E30" t="s">
-        <v>33</v>
-      </c>
-      <c r="F30" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+      <c r="G30" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>2</v>
       </c>
-      <c r="B31" s="4" t="s">
-        <v>55</v>
-      </c>
+      <c r="B31" s="4"/>
       <c r="C31" t="s">
-        <v>14</v>
-      </c>
-      <c r="E31" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
+        <v>187</v>
+      </c>
+      <c r="G31" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>2</v>
       </c>
-      <c r="B32" t="s">
-        <v>56</v>
+      <c r="B32" s="4" t="s">
+        <v>55</v>
       </c>
       <c r="C32" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="E32" t="s">
         <v>33</v>
+      </c>
+      <c r="F32" t="s">
+        <v>39</v>
+      </c>
+      <c r="G32" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
@@ -3284,21 +3598,21 @@
         <v>55</v>
       </c>
       <c r="C33" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E33" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>2</v>
       </c>
-      <c r="B34" s="4" t="s">
-        <v>55</v>
+      <c r="B34" t="s">
+        <v>56</v>
       </c>
       <c r="C34" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E34" t="s">
         <v>33</v>
@@ -3312,7 +3626,7 @@
         <v>55</v>
       </c>
       <c r="C35" t="s">
-        <v>59</v>
+        <v>18</v>
       </c>
       <c r="E35" t="s">
         <v>33</v>
@@ -3326,7 +3640,7 @@
         <v>55</v>
       </c>
       <c r="C36" t="s">
-        <v>58</v>
+        <v>19</v>
       </c>
       <c r="E36" t="s">
         <v>33</v>
@@ -3340,7 +3654,7 @@
         <v>55</v>
       </c>
       <c r="C37" t="s">
-        <v>21</v>
+        <v>59</v>
       </c>
       <c r="E37" t="s">
         <v>33</v>
@@ -3354,7 +3668,7 @@
         <v>55</v>
       </c>
       <c r="C38" t="s">
-        <v>22</v>
+        <v>58</v>
       </c>
       <c r="E38" t="s">
         <v>33</v>
@@ -3368,7 +3682,7 @@
         <v>55</v>
       </c>
       <c r="C39" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E39" t="s">
         <v>33</v>
@@ -3382,7 +3696,7 @@
         <v>55</v>
       </c>
       <c r="C40" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E40" t="s">
         <v>33</v>
@@ -3396,7 +3710,7 @@
         <v>55</v>
       </c>
       <c r="C41" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E41" t="s">
         <v>33</v>
@@ -3410,12 +3724,11 @@
         <v>55</v>
       </c>
       <c r="C42" t="s">
-        <v>48</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F42" s="3"/>
+        <v>24</v>
+      </c>
+      <c r="E42" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43">
@@ -3425,38 +3738,39 @@
         <v>55</v>
       </c>
       <c r="C43" t="s">
-        <v>41</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>31</v>
+        <v>25</v>
+      </c>
+      <c r="E43" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>55</v>
       </c>
       <c r="C44" t="s">
-        <v>57</v>
-      </c>
-      <c r="E44" t="s">
-        <v>33</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F44" s="3"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B45" s="4" t="s">
         <v>55</v>
       </c>
       <c r="C45" t="s">
-        <v>20</v>
-      </c>
-      <c r="E45" t="s">
-        <v>33</v>
+        <v>41</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
@@ -3467,7 +3781,7 @@
         <v>55</v>
       </c>
       <c r="C46" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="E46" t="s">
         <v>33</v>
@@ -3481,10 +3795,10 @@
         <v>55</v>
       </c>
       <c r="C47" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="E47" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
@@ -3495,10 +3809,10 @@
         <v>55</v>
       </c>
       <c r="C48" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E48" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
@@ -3509,13 +3823,10 @@
         <v>55</v>
       </c>
       <c r="C49" t="s">
-        <v>28</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F49" s="3" t="s">
-        <v>60</v>
+        <v>26</v>
+      </c>
+      <c r="E49" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
@@ -3526,10 +3837,10 @@
         <v>55</v>
       </c>
       <c r="C50" t="s">
-        <v>42</v>
-      </c>
-      <c r="E50" s="3" t="s">
-        <v>33</v>
+        <v>27</v>
+      </c>
+      <c r="E50" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
@@ -3540,10 +3851,13 @@
         <v>55</v>
       </c>
       <c r="C51" t="s">
-        <v>43</v>
-      </c>
-      <c r="E51" t="s">
-        <v>47</v>
+        <v>28</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
@@ -3554,10 +3868,10 @@
         <v>55</v>
       </c>
       <c r="C52" t="s">
-        <v>44</v>
-      </c>
-      <c r="E52" t="s">
-        <v>46</v>
+        <v>42</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
@@ -3568,10 +3882,10 @@
         <v>55</v>
       </c>
       <c r="C53" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E53" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
@@ -3582,7 +3896,7 @@
         <v>55</v>
       </c>
       <c r="C54" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E54" t="s">
         <v>46</v>
@@ -3596,9 +3910,37 @@
         <v>55</v>
       </c>
       <c r="C55" t="s">
+        <v>45</v>
+      </c>
+      <c r="E55" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>3</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C56" t="s">
+        <v>49</v>
+      </c>
+      <c r="E56" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>3</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C57" t="s">
         <v>50</v>
       </c>
-      <c r="E55" t="s">
+      <c r="E57" t="s">
         <v>46</v>
       </c>
     </row>
@@ -3611,6 +3953,15 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65D11A73-AFDF-D34A-812F-422461503E72}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8577ECF-3B0E-BA46-812D-AE5953F82593}">
   <dimension ref="B1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3620,10 +3971,10 @@
   <sheetData>
     <row r="1" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C1" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D1" t="s">
         <v>37</v>
@@ -3631,190 +3982,195 @@
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C3" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="D3" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C4" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C5" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C6" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="D6" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="C7" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C8" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D8" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C9" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D9" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C10" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D10" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C11" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D11" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D12" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D13" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D14" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D15" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D16" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D17" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D18" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D19" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D20" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>180</v>
+        <v>176</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>